<commit_message>
feat(F-NAR-009): PAR, EMO.GES et ramifiées AUT-005/006/011/012
Ouvertures descriptives distinctes. Texte seulement.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.002-01.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.002-01.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Noé finit sa phrase</t>
+          <t>Le bateau de Chouchou</t>
         </is>
       </c>
     </row>
@@ -830,6 +830,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Chouchou apporte un dessin. Le papier tremble. Amir connaît le mot. Il attend. Chouchou finit : un bateau bleu, une voile, une mer ronde.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1184,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la cuisine sent le pain chaud. Papa coupe des carottes. Sara est sur sa chaise. Noé arrive avec un dessin. Le papier tremble un peu. Noé veut raconter. J'ai fait.. Puis il cherche le mot. Sara connaît le dessin. Elle veut dire le mot. Elle ouvre la bouche. Papa pose la main, doucement, près de la table. On peut laisser le temps. On n'achève pas à sa place. Sara referme la bouche. Elle attend la fin de la phrase. Noé respire. J'ai fait un bateau. Il est bleu. Noé hoche la tête. Il recommence. Et il y a.. Encore un silence. Sara compte dans sa tête. Un. Deux. Trois. Une voile. Papa sourit. Merci d'avoir su attendre. On peut laisser le temps. Sara pose le dessin contre le sel. Noé s'assoit. Papa donne une rondelle de carotte. Sara croque. Noé croque. Noé dit encore : demain, je veux.. Il s'arrête. Sara attend. Le frigo ronronne. Demain je veux de la peinture. Moi aussi. Ils parlent, un peu lentement. Papa met l'eau dans les verres. On laisse le temps. On écoute jusqu'au bout. Sara répète : jusqu'au bout. Après le repas, Noé montre encore le bateau. La mer est.. Sara attend. La mer est ronde. Sara rit gentiment, sans couper. Le dessin reste sur la table, bien à sa place.</t>
+          <t>La buée dessine des ronds sur la vitre. Derrière les ronds, le village est déjà bleu. L'odeur du pain chaud monte l'escalier. La nappe à carreaux est un peu rêche. Papa coupe des carottes orange, tout doucement. Le pain est encore tiède, Amir. Tu entends le frigo ? Oui, papa. Il ronronne. En ce moment, Amir est sur sa chaise. Ses pieds touchent la barre de bois. La porte de la cuisine s'ouvre un peu. Chouchou arrive avec un papier. Le papier tremble entre ses doigts. Un crayon bleu a laissé une trace. J'ai fait... Chouchou s'arrête. Il cherche le mot. Amir connaît le dessin. C'est un bateau. Amir ouvre la bouche. Le mot est déjà là, tout prêt. On peut laisser le temps, Amir. On attend la fin de la phrase. Amir referme la bouche. Il pose ses mains à plat sur la table. Il compte dans sa tête. Un. Deux. Trois. Le frigo ronronne encore. J'ai fait un bateau. Il est bleu. Chouchou hoche la tête. Et il y a... Encore un silence. Amir attend. Il regarde le sel sur la table. Une voile. Bravo, Amir. Tu as su attendre. C'est du bon travail. Amir pose le dessin contre le pot de sel. Papa donne une rondelle de carotte. Amir croque. C'est un peu sucré. Chouchou croque aussi. Demain, je veux... Il s'arrête encore. Amir attend encore. Une goutte tombe dans l'évier. Demain je veux de la peinture. Moi aussi. Vous parlez bien, l'un après l'autre. Vous avez fini votre rondelle ? Presque, papa. Papa met de l'eau dans les verres. L'eau fait un petit bruit clair. Après le repas, Chouchou montre encore le bateau. La mer est... Amir attend la fin. La mer est ronde. Elle est ronde, oui. Vous avez laissé le temps. On écoute jusqu'au bout. Jusqu'au bout. Le dessin reste sur la table. Il est bien à sa place.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1312,27 +1324,72 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le soir, la cuisine sent le pain chaud. Papa coupe des carottes. Sara est sur sa chaise. Noé arrive avec un dessin. Le papier tremble un peu. Noé veut raconter.
-narrateur|J'ai fait..
-narrateur|Puis il cherche le mot. Sara connaît le dessin. Elle veut dire le mot. Elle ouvre la bouche. Papa pose la main, doucement, près de la table.
-papa|On peut laisser le temps. On n'achève pas à sa place.
-narrateur|Sara referme la bouche. Elle attend la fin de la phrase. Noé respire.
-narrateur|J'ai fait un bateau.
-enfant-f|Il est bleu.
-narrateur|Noé hoche la tête. Il recommence.
-narrateur|Et il y a.. Encore un silence.
-narrateur|Sara compte dans sa tête. Un. Deux. Trois.
-copain|Une voile. Papa sourit.
-papa|Merci d'avoir su attendre. On peut laisser le temps.
-narrateur|Sara pose le dessin contre le sel. Noé s'assoit. Papa donne une rondelle de carotte. Sara croque. Noé croque. Noé dit encore : demain, je veux.. Il s'arrête. Sara attend. Le frigo ronronne.
+          <t>narrateur|La buée dessine des ronds sur la vitre.
+narrateur|Derrière les ronds, le village est déjà bleu.
+narrateur|L'odeur du pain chaud monte l'escalier.
+narrateur|La nappe à carreaux est un peu rêche.
+narrateur|Papa coupe des carottes orange, tout doucement.
+papa|Le pain est encore tiède, Amir.
+papa|Tu entends le frigo ?
+enfant-m|Oui, papa. Il ronronne.
+narrateur|En ce moment, Amir est sur sa chaise.
+narrateur|Ses pieds touchent la barre de bois.
+narrateur|La porte de la cuisine s'ouvre un peu.
+narrateur|Chouchou arrive avec un papier.
+narrateur|Le papier tremble entre ses doigts.
+narrateur|Un crayon bleu a laissé une trace.
+copain|J'ai fait...
+narrateur|Chouchou s'arrête.
+narrateur|Il cherche le mot.
+narrateur|Amir connaît le dessin.
+narrateur|C'est un bateau.
+narrateur|Amir ouvre la bouche.
+narrateur|Le mot est déjà là, tout prêt.
+papa|On peut laisser le temps, Amir.
+papa|On attend la fin de la phrase.
+narrateur|Amir referme la bouche.
+narrateur|Il pose ses mains à plat sur la table.
+narrateur|Il compte dans sa tête.
+narrateur|Un.
+narrateur|Deux.
+narrateur|Trois.
+narrateur|Le frigo ronronne encore.
+copain|J'ai fait un bateau.
+enfant-m|Il est bleu.
+narrateur|Chouchou hoche la tête.
+copain|Et il y a...
+narrateur|Encore un silence.
+narrateur|Amir attend.
+narrateur|Il regarde le sel sur la table.
+copain|Une voile.
+papa|Bravo, Amir.
+papa|Tu as su attendre.
+papa|C'est du bon travail.
+narrateur|Amir pose le dessin contre le pot de sel.
+narrateur|Papa donne une rondelle de carotte.
+narrateur|Amir croque. C'est un peu sucré.
+narrateur|Chouchou croque aussi.
+copain|Demain, je veux...
+narrateur|Il s'arrête encore.
+narrateur|Amir attend encore.
+narrateur|Une goutte tombe dans l'évier.
 copain|Demain je veux de la peinture.
-enfant-f|Moi aussi. Ils parlent, un peu lentement. Papa met l'eau dans les verres.
-narrateur|On laisse le temps. On écoute jusqu'au bout.
-narrateur|Sara répète : jusqu'au bout. Après le repas, Noé montre encore le bateau.
-narrateur|La mer est..
-narrateur|Sara attend.
+enfant-m|Moi aussi.
+papa|Vous parlez bien, l'un après l'autre.
+papa|Vous avez fini votre rondelle ?
+enfant-m|Presque, papa.
+narrateur|Papa met de l'eau dans les verres.
+narrateur|L'eau fait un petit bruit clair.
+narrateur|Après le repas, Chouchou montre encore le bateau.
+copain|La mer est...
+narrateur|Amir attend la fin.
 copain|La mer est ronde.
-narrateur|Sara rit gentiment, sans couper. Le dessin reste sur la table, bien à sa place.</t>
+enfant-m|Elle est ronde, oui.
+papa|Vous avez laissé le temps.
+papa|On écoute jusqu'au bout.
+enfant-m|Jusqu'au bout.
+narrateur|Le dessin reste sur la table.
+narrateur|Il est bien à sa place.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr"/>
@@ -1360,7 +1417,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Noé cherche un mot. Que fait Sara ?</t>
+          <t>Chouchou cherche un mot. Que fait Amir ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1516,7 +1573,7 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Noé cherche un mot. Que fait Sara ?</t>
+          <t>narrateur|Chouchou cherche un mot. Que fait Amir ?</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr"/>
@@ -1544,7 +1601,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sara a su attendre. Noé a fini sa phrase. Papa On peut laisser le temps.</t>
+          <t>Amir a su attendre. Chouchou a fini sa phrase. On peut laisser le temps. Tu as attendu la fin, Amir. J'ai laissé le temps. Bravo. C'est du bon travail. Le bateau bleu reste contre le sel.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1688,8 +1745,13 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sara a su attendre. Noé a fini sa phrase. Papa
-enfant-f|On peut laisser le temps.</t>
+          <t>narrateur|Amir a su attendre.
+narrateur|Chouchou a fini sa phrase.
+papa|On peut laisser le temps.
+papa|Tu as attendu la fin, Amir.
+enfant-m|J'ai laissé le temps.
+papa|Bravo. C'est du bon travail.
+narrateur|Le bateau bleu reste contre le sel.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr"/>
@@ -1717,7 +1779,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Papa range les assiettes. Sara donne le dessin à Noé. Noé le tient tout seul. Ils vont vers le salon.</t>
+          <t>Papa range les assiettes. Elles font un petit bruit doux. Tu donnes le dessin à Chouchou ? Oui, papa. Amir donne le dessin. Chouchou le tient tout seul. On va vers le salon ? Oui. Ils marchent sans se presser. La cuisine sent encore le pain.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1853,7 +1915,16 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Papa range les assiettes. Sara donne le dessin à Noé. Noé le tient tout seul. Ils vont vers le salon.</t>
+          <t>narrateur|Papa range les assiettes.
+narrateur|Elles font un petit bruit doux.
+papa|Tu donnes le dessin à Chouchou ?
+enfant-m|Oui, papa.
+narrateur|Amir donne le dessin.
+narrateur|Chouchou le tient tout seul.
+papa|On va vers le salon ?
+copain|Oui.
+narrateur|Ils marchent sans se presser.
+narrateur|La cuisine sent encore le pain.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr"/>
@@ -1881,7 +1952,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>J'ai attendu la fin. Bravo, Amir. Tu as fait du bon travail. Le bateau bleu reste dans la main de Chouchou. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2021,7 +2092,11 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>enfant-m|J'ai attendu la fin.
+papa|Bravo, Amir.
+papa|Tu as fait du bon travail.
+narrateur|Le bateau bleu reste dans la main de Chouchou.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr"/>
@@ -2043,7 +2118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2081,6 +2156,20 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.002-01 Nino finit sa phrase
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.002-01.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.002-01.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le bateau de Chouchou</t>
+          <t>Nino finit sa phrase</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine</t>
+          <t>maison, cuisine, soir, pain, carottes, dessin, papier, crayon bleu, table, lampe</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Amir, Chouchou, papa</t>
+          <t>Sarah, Nino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chouchou apporte un dessin. Le papier tremble. Amir connaît le mot. Il attend. Chouchou finit : un bateau bleu, une voile, une mer ronde.</t>
+          <t>La vitre orange tient le soir. Près du pain, un éclat de carotte brille. Sarah veut montrer le dessin, maintenant. Nino cherche un mot. Elle ouvre la bouche trop vite, pousse le papier. Sourire parti, poitrine, papa accroupi. Elle refuse de foncer, referme la bouche, attend. Nino finit. Merci vécu. Deuxième ruse : une voile. Un éclat de carotte tient près du pain.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La buée dessine des ronds sur la vitre. Derrière les ronds, le village est déjà bleu. L'odeur du pain chaud monte l'escalier. La nappe à carreaux est un peu rêche. Papa coupe des carottes orange, tout doucement. Le pain est encore tiède, Amir. Tu entends le frigo ? Oui, papa. Il ronronne. En ce moment, Amir est sur sa chaise. Ses pieds touchent la barre de bois. Une miette de pain dort près de l'assiette. Tu veux un coin de croûte ? Oui. Elle est tiède. Amir croque. La croûte craque un peu. La porte de la cuisine s'ouvre un peu. Chouchou arrive avec un papier. Le papier tremble entre ses doigts. Un crayon bleu a laissé une trace. J'ai fait... Chouchou s'arrête. Il cherche le mot. Amir connaît le dessin. C'est un bateau. Amir ouvre la bouche. Le mot est déjà là, tout prêt. On peut laisser le temps, Amir. On attend la fin de la phrase. Amir referme la bouche. Il pose ses mains à plat sur la table. Il compte dans sa tête. Un. Deux. Trois. Le frigo ronronne encore. J'ai fait un bateau. Il est bleu. Chouchou hoche la tête. Et il y a... Encore un silence. Amir attend. Il regarde le sel sur la table. Une voile. Bravo, Amir. Tu as su attendre. Amir pose le dessin contre le pot de sel. Papa donne une rondelle de carotte. Amir croque. C'est un peu sucré. Chouchou croque aussi. Demain, je veux... Il s'arrête encore. Amir attend encore. Une goutte tombe dans l'évier. Demain je veux de la peinture. Moi aussi. Vous parlez bien, l'un après l'autre. Vous avez fini votre rondelle ? Presque, papa. Papa met de l'eau dans les verres. L'eau fait un petit bruit clair. Après le repas, Chouchou montre encore le bateau. La mer est... Amir attend la fin. La mer est ronde. Elle est ronde, oui. Vous avez laissé le temps. On écoute jusqu'au bout. Jusqu'au bout. Le dessin reste sur la table. Il est bien à sa place.</t>
+          <t>La vitre orange tient le soir dehors. L'odeur du pain chaud remplit la cuisine. Ça sent bon, papa. Tu le sens, le pain, Sarah ? Oui, papa. Papa coupe des carottes orange. Une rondelle tombe près du pain. Elle est orange, maman. Tu la vois, la rondelle ? Oui, maman. Près du pain, un éclat de carotte brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Maman casse le pain. La croûte craque, tiède. Elle est tiède. Tu veux un coin de croûte ? Oui. Sarah croque. La croûte gratte un peu. Le pain tient chaud, Sarah ? Oui, papa. En ce moment, Sarah tient un papier. Un crayon bleu a laissé une trace. Je veux montrer le dessin, maintenant ! Sur la table, tout de suite. Le dessin, là ? Oui, le dessin. Tes mains tiennent le papier, Sarah ? Oui, maman. La porte s'ouvre. Nino arrive avec un papier. Le papier tremble entre ses doigts. Je le montre, maintenant ! Sarah prend le papier trop vite. J'ai fait. Nino s'arrête. Il cherche le mot. Sarah connaît le dessin. C'est un bateau. Les mots montent très vite. Le bateau ! La voile ! Maintenant ! Sarah pousse le papier trop vite. Le papier tape le pain. Oh. Le dessin glisse vers l'éclat. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Sarah ? Oui, papa. Le papier est près du pain, Sarah ? Un peu, maman. L'éclat de carotte tremble, puis tient. Nino baisse les yeux. Il ne dit plus le mot, papa. Sarah regarde papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La buée dessine des ronds sur la vitre. Derrière les ronds, le village est déjà bleu. L'odeur du pain chaud monte l'escalier. La nappe à carreaux est un peu rêche. Papa coupe des carottes orange, tout doucement. Le pain est encore tiède, Amir. Tu entends le frigo ? Oui, papa. Il ronronne. En ce moment, Amir est sur sa chaise. Ses pieds touchent la barre de bois. Une miette de pain dort près de l'assiette. Tu veux un coin de croûte ? Oui. Elle est tiède. Amir croque. La croûte craque un peu. La porte de la cuisine s'ouvre un peu. Chouchou arrive avec un papier. Le papier tremble entre ses doigts. Un crayon bleu a laissé une trace. J'ai fait... Chouchou s'arrête. Il cherche le mot. Amir connaît le dessin. C'est un bateau. Amir ouvre la bouche. Le mot est déjà là, tout prêt. On peut laisser le temps, Amir. On attend la fin de la phrase. Amir referme la bouche. Il pose ses mains à plat sur la table. Il compte dans sa tête. Un. Deux. Trois. Le frigo ronronne encore. J'ai fait un bateau. Il est bleu. Chouchou hoche la tête. Et il y a... Encore un silence. Amir attend. Il regarde le sel sur la table. Une voile. Bravo, Amir. Tu as su attendre. Amir pose le dessin contre le pot de sel. Papa donne une rondelle de carotte. Amir croque. C'est un peu sucré. Chouchou croque aussi. Demain, je veux... Il s'arrête encore. Amir attend encore. Une goutte tombe dans l'évier. Demain je veux de la peinture. Moi aussi. Vous parlez bien, l'un après l'autre. Vous avez fini votre rondelle ? Presque, papa. Papa met de l'eau dans les verres. L'eau fait un petit bruit clair. Après le repas, Chouchou montre encore le bateau. La mer est... Amir attend la fin. La mer est ronde. Elle est ronde, oui. Vous avez laissé le temps. On écoute jusqu'au bout. Jusqu'au bout. Le dessin reste sur la table. Il est bien à sa place.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La vitre orange tient le soir dehors. L'odeur du pain chaud remplit la cuisine. Ça sent bon, papa. Tu le sens, le pain, Sarah ? Oui, papa. Papa coupe des carottes orange. Une rondelle tombe près du pain. Elle est orange, maman. Tu la vois, la rondelle ? Oui, maman. Près du pain, un &lt;emphasis level="moderate"&gt;éclat de carotte&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Maman casse le pain. La croûte craque, tiède. Elle est tiède. Tu veux un coin de croûte ? Oui. Sarah croque. La croûte gratte un peu. Le pain tient chaud, Sarah ? Oui, papa. En ce moment, Sarah tient un papier. Un crayon bleu a laissé une trace. Je veux montrer le dessin, maintenant ! Sur la table, tout de suite. Le dessin, là ? Oui, le dessin. Tes mains tiennent le papier, Sarah ? Oui, maman. La porte s'ouvre. Nino arrive avec un papier. Le papier tremble entre ses doigts. Je le montre, maintenant ! Sarah prend le papier trop vite. J'ai fait. Nino s'arrête. Il cherche le mot. Sarah connaît le dessin. C'est un bateau. Les mots montent très vite. Le bateau ! La voile ! Maintenant ! Sarah pousse le papier trop vite. Le papier tape le pain. Oh. Le dessin glisse vers l'éclat. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Sarah ? Oui, papa. Le papier est près du pain, Sarah ? Un peu, maman. L'éclat de carotte tremble, puis tient. Nino baisse les yeux. Il ne dit plus le mot, papa. Sarah regarde papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la cuisine sent le pain chaud. Papa coupe des carottes. Sara est sur sa chaise. Noé arrive avec un dessin. Le papier tremble un peu. Noé veut raconter. Il dit : j'ai fait.. Puis il cherche le mot. Sara connaît le dessin. Elle veut dire le mot. Elle ouvre la bouche. Papa pose la main, doucement, près de la table. Papa dit : on peut &lt;emphasis&gt;laisser&lt;/emphasis&gt; le temps. On n'achève pas à sa place. Sara referme la bouche. Elle attend la fin de la phrase. Noé respire. Il dit : j'ai fait un bateau. Sara dit : il est bleu. Noé hoche la tête. Il recommence. Il dit : et il y a.. Encore un silence. Sara compte dans sa tête. Un. Deux. Trois. Noé dit : une voile. Papa sourit. Papa dit : merci d'avoir su attendre. On peut laisser le temps. Sara pose le dessin contre le sel. Noé s'assoit. Papa donne une rondelle de carotte. Sara croque. Noé croque. Noé dit encore : demain, je veux.. Il s'arrête. Sara attend. Le frigo ronronne. Noé dit : demain je veux de la peinture. Sara dit : moi aussi. Ils parlent, un peu lentement. Papa met l'eau dans les verres. Il dit : on laisse le temps. On écoute jusqu'au bout. Sara répète : jusqu'au bout. Après le repas, Noé montre encore le bateau. Il dit : la mer est.. Sara attend. Noé dit : la mer est ronde. Sara rit gentiment, sans couper. Le dessin reste sur la table, bien à sa place. [pause]</t>
+          <t>La vitre orange tient le soir dehors. L'odeur du pain chaud remplit la cuisine. Ça sent bon, papa. Tu le sens, le pain, Sarah ? Oui, papa. Papa coupe des carottes orange. Une rondelle tombe près du pain. Elle est orange, maman. Tu la vois, la rondelle ? Oui, maman. Près du pain, un &lt;emphasis&gt;éclat de carotte&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Maman casse le pain. La croûte craque, tiède. Elle est tiède. Tu veux un coin de croûte ? Oui. Sarah croque. La croûte gratte un peu. Le pain tient chaud, Sarah ? Oui, papa. En ce moment, Sarah tient un papier. Un crayon bleu a laissé une trace. Je veux montrer le dessin, maintenant ! Sur la table, tout de suite. Le dessin, là ? Oui, le dessin. Tes mains tiennent le papier, Sarah ? Oui, maman. La porte s'ouvre. Nino arrive avec un papier. Le papier tremble entre ses doigts. Je le montre, maintenant ! Sarah prend le papier trop vite. J'ai fait. Nino s'arrête. Il cherche le mot. Sarah connaît le dessin. C'est un bateau. Les mots montent très vite. Le bateau ! La voile ! Maintenant ! Sarah pousse le papier trop vite. Le papier tape le pain. Oh. Le dessin glisse vers l'éclat. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Sarah ? Oui, papa. Le papier est près du pain, Sarah ? Un peu, maman. L'éclat de carotte tremble, puis tient. Nino baisse les yeux. Il ne dit plus le mot, papa. Sarah regarde papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>laisser</t>
+          <t>éclat de carotte</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,82 +1321,79 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_montrer_le_dessin_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La buée dessine des ronds sur la vitre.
-narrateur|Derrière les ronds, le village est déjà bleu.
-narrateur|L'odeur du pain chaud monte l'escalier.
-narrateur|La nappe à carreaux est un peu rêche.
-narrateur|Papa coupe des carottes orange, tout doucement.
-papa|Le pain est encore tiède, Amir.
-papa|Tu entends le frigo ?
-enfant-m|Oui, papa.
-enfant-m|Il ronronne.
-narrateur|En ce moment, Amir est sur sa chaise.
-narrateur|Ses pieds touchent la barre de bois.
-narrateur|Une miette de pain dort près de l'assiette.
-papa|Tu veux un coin de croûte ?
-enfant-m|Oui.
-enfant-m|Elle est tiède.
-narrateur|Amir croque.
-narrateur|La croûte craque un peu.
-narrateur|La porte de la cuisine s'ouvre un peu.
-narrateur|Chouchou arrive avec un papier.
+          <t>narrateur|La vitre orange tient le soir dehors.
+narrateur|L'odeur du pain chaud remplit la cuisine.
+enfant-f|Ça sent bon, papa.
+papa|Tu le sens, le pain, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Papa coupe des carottes orange.
+narrateur|Une rondelle tombe près du pain.
+enfant-f|Elle est orange, maman.
+maman|Tu la vois, la rondelle ?
+enfant-f|Oui, maman.
+narrateur|Près du pain, un éclat de carotte brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Maman casse le pain.
+narrateur|La croûte craque, tiède.
+enfant-f|Elle est tiède.
+maman|Tu veux un coin de croûte ?
+enfant-f|Oui.
+narrateur|Sarah croque.
+narrateur|La croûte gratte un peu.
+papa|Le pain tient chaud, Sarah ?
+enfant-f|Oui, papa.
+narrateur|En ce moment, Sarah tient un papier.
+narrateur|Un crayon bleu a laissé une trace.
+enfant-f|Je veux montrer le dessin, maintenant !
+enfant-f|Sur la table, tout de suite.
+papa|Le dessin, là ?
+enfant-f|Oui, le dessin.
+maman|Tes mains tiennent le papier, Sarah ?
+enfant-f|Oui, maman.
+narrateur|La porte s'ouvre.
+narrateur|Nino arrive avec un papier.
 narrateur|Le papier tremble entre ses doigts.
-narrateur|Un crayon bleu a laissé une trace.
-copain|J'ai fait...
-narrateur|Chouchou s'arrête.
+enfant-f|Je le montre, maintenant !
+narrateur|Sarah prend le papier trop vite.
+copain|J'ai fait.
+narrateur|Nino s'arrête.
 narrateur|Il cherche le mot.
-narrateur|Amir connaît le dessin.
+narrateur|Sarah connaît le dessin.
 narrateur|C'est un bateau.
-narrateur|Amir ouvre la bouche.
-narrateur|Le mot est déjà là, tout prêt.
-papa|On peut laisser le temps, Amir.
-papa|On attend la fin de la phrase.
-narrateur|Amir referme la bouche.
-narrateur|Il pose ses mains à plat sur la table.
-narrateur|Il compte dans sa tête.
-narrateur|Un.
-narrateur|Deux.
-narrateur|Trois.
-narrateur|Le frigo ronronne encore.
-copain|J'ai fait un bateau.
-enfant-m|Il est bleu.
-narrateur|Chouchou hoche la tête.
-copain|Et il y a...
-narrateur|Encore un silence.
-narrateur|Amir attend.
-narrateur|Il regarde le sel sur la table.
-copain|Une voile.
-papa|Bravo, Amir.
-papa|Tu as su attendre.
-narrateur|Amir pose le dessin contre le pot de sel.
-narrateur|Papa donne une rondelle de carotte.
-narrateur|Amir croque.
-narrateur|C'est un peu sucré.
-narrateur|Chouchou croque aussi.
-copain|Demain, je veux...
-narrateur|Il s'arrête encore.
-narrateur|Amir attend encore.
-narrateur|Une goutte tombe dans l'évier.
-copain|Demain je veux de la peinture.
-enfant-m|Moi aussi.
-papa|Vous parlez bien, l'un après l'autre.
-papa|Vous avez fini votre rondelle ?
-enfant-m|Presque, papa.
-narrateur|Papa met de l'eau dans les verres.
-narrateur|L'eau fait un petit bruit clair.
-narrateur|Après le repas, Chouchou montre encore le bateau.
-copain|La mer est...
-narrateur|Amir attend la fin.
-copain|La mer est ronde.
-enfant-m|Elle est ronde, oui.
-papa|Vous avez laissé le temps.
-papa|On écoute jusqu'au bout.
-enfant-m|Jusqu'au bout.
-narrateur|Le dessin reste sur la table.
-narrateur|Il est bien à sa place.</t>
+narrateur|Les mots montent très vite.
+enfant-f|Le bateau !
+enfant-f|La voile !
+enfant-f|Maintenant !
+narrateur|Sarah pousse le papier trop vite.
+narrateur|Le papier tape le pain.
+enfant-f|Oh.
+narrateur|Le dessin glisse vers l'éclat.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Nino, Sarah ?
+enfant-f|Oui, papa.
+maman|Le papier est près du pain, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de carotte tremble, puis tient.
+narrateur|Nino baisse les yeux.
+enfant-f|Il ne dit plus le mot, papa.
+narrateur|Sarah regarde papa.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>pain</t>
         </is>
       </c>
     </row>
@@ -1423,17 +1420,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou cherche un mot. Que fait Amir ?</t>
+          <t>Nino cherche un mot. Que fait Sarah ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou cherche un mot. Que fait Amir ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino cherche un mot. Que fait &lt;emphasis level="moderate"&gt;Sarah&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Noé cherche un mot. Que fait Sara ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino cherche un mot. Que fait &lt;emphasis&gt;Sarah&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1496,7 +1493,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1507,7 +1504,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1522,34 +1519,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Sarah</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1564,23 +1565,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=nino_cherche_un_mot_que_fait_sarah; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou cherche un mot.
-narrateur|Que fait Amir ?</t>
+          <t>narrateur|Nino cherche un mot.
+narrateur|Que fait Sarah ?</t>
         </is>
       </c>
     </row>
@@ -1607,17 +1608,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir a su attendre. Chouchou a fini sa phrase. On peut laisser le temps. Tu as attendu la fin, Amir. J'ai laissé le temps. Bravo. Le bateau bleu reste contre le sel.</t>
+          <t>Sarah veut montrer le dessin, tout de suite. Je le dis, maintenant ! Elle ouvre la bouche. Les mots se bousculent dans sa bouche. Nino baisse les yeux. Il serre le bord du papier. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le dessin, un instant. Elle écoute le silence de la cuisine. Tu veux montrer le dessin avec Nino ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le papier, puis on reste. D'accord. Sarah reste un moment, les mains ouvertes. Elle attend. J'ai fait un bateau. Il est bleu. Nino hoche la tête. Sarah pose le dessin contre le sel. Merci, Sarah. Papa a vu les deux, à la cuisine. La croûte est tiède, sous les doigts. Elle est chaude. Papa donne une rondelle de carotte. Sarah croque. C'est un peu sucré. Nino croque aussi. Le bateau. Il a une voile, là ? Oui, là. Sarah glisse la main sur le papier. Le crayon est lisse, contre la peau. Tes mains sont au chaud, Sarah ? Un peu, maman. Nino pose un doigt sur la voile. Bleu. On le laisse sur la table ? Le pain est près du dessin. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir a su attendre. Chouchou a fini sa phrase. On peut laisser le temps. Tu as attendu la fin, Amir. J'ai laissé le temps. Bravo. Le bateau bleu reste contre le sel.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah veut montrer le dessin, tout de suite. Je le dis, maintenant ! Elle ouvre la bouche. Les mots se bousculent dans sa bouche. Nino baisse les yeux. Il serre le bord du papier. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le dessin, un instant. Elle écoute le silence de la cuisine. Tu veux montrer le dessin avec Nino ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le papier, puis on reste. D'accord. Sarah reste un moment, les mains ouvertes. Elle attend. J'ai fait un &lt;emphasis level="moderate"&gt;bateau&lt;/emphasis&gt;. Il est bleu. Nino hoche la tête. Sarah pose le dessin contre le sel. Merci, Sarah. Papa a vu les deux, à la cuisine. La croûte est tiède, sous les doigts. Elle est chaude. Papa donne une rondelle de carotte. Sarah croque. C'est un peu sucré. Nino croque aussi. Le bateau. Il a une voile, là ? Oui, là. Sarah glisse la main sur le papier. Le crayon est lisse, contre la peau. Tes mains sont au chaud, Sarah ? Un peu, maman. Nino pose un doigt sur la voile. Bleu. On le laisse sur la table ? Le pain est près du dessin. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Sara a su attendre. Noé a fini sa phrase. Papa a dit : on peut &lt;emphasis&gt;laisser&lt;/emphasis&gt; le temps. [pause]</t>
+          <t>Sarah veut montrer le dessin, tout de suite. Je le dis, maintenant ! Elle ouvre la bouche. Les mots se bousculent dans sa bouche. Nino baisse les yeux. Il serre le bord du papier. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le dessin, un instant. Elle écoute le silence de la cuisine. Tu veux montrer le dessin avec Nino ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le papier, puis on reste. D'accord. Sarah reste un moment, les mains ouvertes. Elle attend. J'ai fait un &lt;emphasis&gt;bateau&lt;/emphasis&gt;. Il est bleu. Nino hoche la tête. Sarah pose le dessin contre le sel. Merci, Sarah. Papa a vu les deux, à la cuisine. La croûte est tiède, sous les doigts. Elle est chaude. Papa donne une rondelle de carotte. Sarah croque. C'est un peu sucré. Nino croque aussi. Le bateau. Il a une voile, là ? Oui, là. Sarah glisse la main sur le papier. Le crayon est lisse, contre la peau. Tes mains sont au chaud, Sarah ? Un peu, maman. Nino pose un doigt sur la voile. Bleu. On le laisse sur la table ? Le pain est près du dessin. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1664,7 +1665,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1672,10 +1673,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1698,30 +1699,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>laisser</t>
+          <t>bateau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1730,10 +1731,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1746,18 +1747,60 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_ouvre_referme_attend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir a su attendre.
-narrateur|Chouchou a fini sa phrase.
-papa|On peut laisser le temps.
-papa|Tu as attendu la fin, Amir.
-enfant-m|J'ai laissé le temps.
-papa|Bravo.
-narrateur|Le bateau bleu reste contre le sel.</t>
+          <t>narrateur|Sarah veut montrer le dessin, tout de suite.
+enfant-f|Je le dis, maintenant !
+narrateur|Elle ouvre la bouche.
+narrateur|Les mots se bousculent dans sa bouche.
+narrateur|Nino baisse les yeux.
+narrateur|Il serre le bord du papier.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Sarah refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe le dessin, un instant.
+narrateur|Elle écoute le silence de la cuisine.
+papa|Tu veux montrer le dessin avec Nino ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Papa, on fait quoi ?
+papa|On pose le papier, puis on reste.
+enfant-f|D'accord.
+narrateur|Sarah reste un moment, les mains ouvertes.
+narrateur|Elle attend.
+copain|J'ai fait un bateau.
+enfant-f|Il est bleu.
+narrateur|Nino hoche la tête.
+narrateur|Sarah pose le dessin contre le sel.
+papa|Merci, Sarah.
+narrateur|Papa a vu les deux, à la cuisine.
+maman|La croûte est tiède, sous les doigts.
+enfant-f|Elle est chaude.
+narrateur|Papa donne une rondelle de carotte.
+narrateur|Sarah croque.
+narrateur|C'est un peu sucré.
+narrateur|Nino croque aussi.
+enfant-f|Le bateau.
+papa|Il a une voile, là ?
+enfant-f|Oui, là.
+narrateur|Sarah glisse la main sur le papier.
+narrateur|Le crayon est lisse, contre la peau.
+maman|Tes mains sont au chaud, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|Nino pose un doigt sur la voile.
+copain|Bleu.
+enfant-f|On le laisse sur la table ?
+maman|Le pain est près du dessin.
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>carotte</t>
         </is>
       </c>
     </row>
@@ -1784,17 +1827,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Papa range les assiettes. Elles font un petit bruit doux. Tu donnes le dessin à Chouchou ? Oui, papa. Amir donne le dessin. Chouchou le tient tout seul. On va vers le salon ? Oui. Ils marchent sans se presser. La cuisine sent encore le pain.</t>
+          <t>Ils restent près de la table. Nino reprend le papier. Et il y a. Une voile, maintenant ! Sarah ouvre la bouche trop vite. Nino serre les lèvres. Oh. Sarah avance les mots, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Sa bouche se ferme, puis s'ouvre. Personne ne dit la suite. Elle observe le dessin, un instant. Elle écoute le silence du pain. Près du pain, un éclat de carotte luit. Là, sur la table. Tu dis le mot, Nino ? Nino ne dit rien. Il tient le papier, sans parler. Une voile. Sarah referme la bouche, sans se presser. Nino pose le papier, plus lentement. Le crayon est lisse et tiède. Tu la vois, la voile ? Oui, papa. Le dessin est près du pain ? Oui, maman. Le bateau tient contre le sel. Sarah pose une main sur le papier. Nino pose la suivante. Le dessin tient, Sarah ? Oui, papa. La lampe passe sur le pain. Elle allume la croûte.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Papa range les assiettes. Elles font un petit bruit doux. Tu donnes le dessin à Chouchou ? Oui, papa. Amir donne le dessin. Chouchou le tient tout seul. On va vers le salon ? Oui. Ils marchent sans se presser. La cuisine sent encore le pain.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent près de la table. Nino reprend le papier. Et il y a. Une voile, maintenant ! Sarah ouvre la bouche trop vite. Nino serre les lèvres. Oh. Sarah avance les mots, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Sa bouche se ferme, puis s'ouvre. Personne ne dit la suite. Elle observe le dessin, un instant. Elle écoute le silence du pain. Près du pain, un &lt;emphasis level="moderate"&gt;éclat de carotte&lt;/emphasis&gt; luit. Là, sur la table. Tu dis le mot, Nino ? Nino ne dit rien. Il tient le papier, sans parler. Une voile. Sarah referme la bouche, sans se presser. Nino pose le papier, plus lentement. Le crayon est lisse et tiède. Tu la vois, la voile ? Oui, papa. Le dessin est près du pain ? Oui, maman. Le bateau tient contre le sel. Sarah pose une main sur le papier. Nino pose la suivante. Le dessin tient, Sarah ? Oui, papa. La lampe passe sur le pain. Elle allume la croûte.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Papa range les assiettes. Sara donne le dessin à Noé. Noé le tient tout seul. Ils vont vers le salon. [pause]</t>
+          <t>Ils restent près de la table. Nino reprend le papier. Et il y a. Une voile, maintenant ! Sarah ouvre la bouche trop vite. Nino serre les lèvres. Oh. Sarah avance les mots, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Sa bouche se ferme, puis s'ouvre. Personne ne dit la suite. Elle observe le dessin, un instant. Elle écoute le silence du pain. Près du pain, un &lt;emphasis&gt;éclat de carotte&lt;/emphasis&gt; luit. Là, sur la table. Tu dis le mot, Nino ? Nino ne dit rien. Il tient le papier, sans parler. Une voile. Sarah referme la bouche, sans se presser. Nino pose le papier, plus lentement. Le crayon est lisse et tiède. Tu la vois, la voile ? Oui, papa. Le dessin est près du pain ? Oui, maman. Le bateau tient contre le sel. Sarah pose une main sur le papier. Nino pose la suivante. Le dessin tient, Sarah ? Oui, papa. La lampe passe sur le pain. Elle allume la croûte. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1841,7 +1884,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1849,10 +1892,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1873,28 +1916,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de carotte</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1903,10 +1950,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1917,19 +1964,52 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=voile_trop_vite_elle_referme_la_bouche; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Papa range les assiettes.
-narrateur|Elles font un petit bruit doux.
-papa|Tu donnes le dessin à Chouchou ?
-enfant-m|Oui, papa.
-narrateur|Amir donne le dessin.
-narrateur|Chouchou le tient tout seul.
-papa|On va vers le salon ?
-copain|Oui.
-narrateur|Ils marchent sans se presser.
-narrateur|La cuisine sent encore le pain.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|Nino reprend le papier.
+copain|Et il y a.
+enfant-f|Une voile, maintenant !
+narrateur|Sarah ouvre la bouche trop vite.
+narrateur|Nino serre les lèvres.
+enfant-f|Oh.
+narrateur|Sarah avance les mots, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Sarah refuse de foncer, cette fois.
+narrateur|Sa bouche se ferme, puis s'ouvre.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le dessin, un instant.
+narrateur|Elle écoute le silence du pain.
+narrateur|Près du pain, un éclat de carotte luit.
+enfant-f|Là, sur la table.
+enfant-f|Tu dis le mot, Nino ?
+narrateur|Nino ne dit rien.
+narrateur|Il tient le papier, sans parler.
+copain|Une voile.
+narrateur|Sarah referme la bouche, sans se presser.
+narrateur|Nino pose le papier, plus lentement.
+narrateur|Le crayon est lisse et tiède.
+papa|Tu la vois, la voile ?
+enfant-f|Oui, papa.
+maman|Le dessin est près du pain ?
+enfant-f|Oui, maman.
+narrateur|Le bateau tient contre le sel.
+narrateur|Sarah pose une main sur le papier.
+narrateur|Nino pose la suivante.
+papa|Le dessin tient, Sarah ?
+enfant-f|Oui, papa.
+maman|La lampe passe sur le pain.
+enfant-f|Elle allume la croûte.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>pain</t>
         </is>
       </c>
     </row>
@@ -1956,17 +2036,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo, Amir. Le bateau bleu reste dans la main de Chouchou.</t>
+          <t>Ils restent près du pain. Le bateau est arrivé, Sarah ? Oui, maman. Tu souffles un peu ? Oui, papa. Sarah souffle, un filet d'air. Le pain sent bon. Tu le sens, le pain ? Oui, maman. La voile reste un peu, bleue. Elle a tenu, sur le papier. Bateau. Le pain est chaud, sous les mains. Le dessin bleu fait de l'ombre. On le montre, après. Un éclat de carotte tient près du pain.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo, Amir. Le bateau bleu reste dans la main de Chouchou.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du pain. Le bateau est arrivé, Sarah ? Oui, maman. Tu souffles un peu ? Oui, papa. Sarah souffle, un filet d'air. Le pain sent bon. Tu le sens, le pain ? Oui, maman. La voile reste un peu, bleue. Elle a tenu, sur le papier. Bateau. Le pain est chaud, sous les mains. Le dessin bleu fait de l'ombre. On le montre, après. Un &lt;emphasis level="moderate"&gt;éclat de carotte&lt;/emphasis&gt; tient près du pain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du pain. Le bateau est arrivé, Sarah ? Oui, maman. Tu souffles un peu ? Oui, papa. Sarah souffle, un filet d'air. Le pain sent bon. Tu le sens, le pain ? Oui, maman. La voile reste un peu, bleue. Elle a tenu, sur le papier. Bateau. Le pain est chaud, sous les mains. Le dessin bleu fait de l'ombre. On le montre, après. Un &lt;emphasis&gt;éclat de carotte&lt;/emphasis&gt; tient près du pain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2013,7 +2093,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2021,10 +2101,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2033,12 +2113,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2047,17 +2127,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de carotte</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2066,11 +2150,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2079,26 +2163,43 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pres_du_pain; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai attendu la fin.
-papa|Bravo, Amir.
-narrateur|Le bateau bleu reste dans la main de Chouchou.</t>
+          <t>narrateur|Ils restent près du pain.
+maman|Le bateau est arrivé, Sarah ?
+enfant-f|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-f|Oui, papa.
+narrateur|Sarah souffle, un filet d'air.
+enfant-f|Le pain sent bon.
+maman|Tu le sens, le pain ?
+enfant-f|Oui, maman.
+papa|La voile reste un peu, bleue.
+enfant-f|Elle a tenu, sur le papier.
+copain|Bateau.
+narrateur|Le pain est chaud, sous les mains.
+narrateur|Le dessin bleu fait de l'ombre.
+enfant-f|On le montre, après.
+narrateur|Un éclat de carotte tient près du pain.</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2183,6 +2284,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>